<commit_message>
add float type check block
Now 12 left blocks
</commit_message>
<xml_diff>
--- a/test/OpenCSTL.xlsx
+++ b/test/OpenCSTL.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\spring\Documents\GitHub\OpenCSTL\test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{518410F7-6DC0-4908-B8FF-B6284058C9A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{520E84C9-2400-4FC6-B6F2-D23AA903792C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4035" yWindow="3870" windowWidth="28800" windowHeight="17190" xr2:uid="{619C67F7-00F0-4C46-A399-483E9C62B008}"/>
+    <workbookView xWindow="1185" yWindow="5745" windowWidth="32055" windowHeight="17190" xr2:uid="{619C67F7-00F0-4C46-A399-483E9C62B008}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="51">
   <si>
     <t>root</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -193,9 +193,6 @@
     <t>base</t>
   </si>
   <si>
-    <t>header(void*)</t>
-  </si>
-  <si>
     <t>compare func</t>
   </si>
   <si>
@@ -212,13 +209,28 @@
   </si>
   <si>
     <t>type_key</t>
+  </si>
+  <si>
+    <t>is_float_key</t>
+  </si>
+  <si>
+    <t>is_float_value</t>
+  </si>
+  <si>
+    <t>arena</t>
+  </si>
+  <si>
+    <t>freelist</t>
+  </si>
+  <si>
+    <t>header(void*) - 8byte</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -235,29 +247,29 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
+      <sz val="14"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="3"/>
+      <name val="KoPubWorld돋움체 Bold"/>
       <charset val="129"/>
-      <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="KoPubWorld돋움체 Bold"/>
       <charset val="129"/>
-      <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
+      <sz val="14"/>
+      <color rgb="FFFF0000"/>
+      <name val="KoPubWorld돋움체 Bold"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <sz val="14"/>
       <color theme="4"/>
-      <name val="Calibri"/>
-      <family val="2"/>
+      <name val="KoPubWorld돋움체 Bold"/>
       <charset val="129"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="7">
@@ -298,7 +310,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -332,56 +344,82 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -698,440 +736,469 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FE06D03-E65E-4121-BF89-D913E6F20D39}">
-  <dimension ref="A1:O14"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:Q14"/>
+  <sheetFormatPr defaultRowHeight="23.25"/>
   <cols>
-    <col min="1" max="1" width="26.7109375" customWidth="1"/>
-    <col min="3" max="3" width="33.85546875" customWidth="1"/>
-    <col min="4" max="4" width="19.28515625" customWidth="1"/>
-    <col min="6" max="6" width="19.28515625" customWidth="1"/>
-    <col min="7" max="7" width="13.7109375" customWidth="1"/>
-    <col min="8" max="8" width="14" customWidth="1"/>
-    <col min="9" max="9" width="14.5703125" customWidth="1"/>
-    <col min="10" max="10" width="16.28515625" customWidth="1"/>
+    <col min="1" max="1" width="34.28515625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="17.28515625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="46.28515625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="19.28515625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="16.5703125" style="1" customWidth="1"/>
+    <col min="6" max="7" width="19.28515625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="23.5703125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="19.42578125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="16.28515625" style="1" customWidth="1"/>
+    <col min="11" max="11" width="19.42578125" style="1" customWidth="1"/>
+    <col min="12" max="12" width="16.42578125" style="1" customWidth="1"/>
+    <col min="13" max="13" width="16.85546875" style="1" customWidth="1"/>
+    <col min="14" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15">
-      <c r="A1" s="1"/>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-    </row>
-    <row r="2" spans="1:15">
-      <c r="C2" s="10" t="s">
+    <row r="1" spans="1:17" s="1" customFormat="1">
+      <c r="A1" s="16"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
+      <c r="K1" s="16"/>
+    </row>
+    <row r="2" spans="1:17" s="1" customFormat="1">
+      <c r="C2" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
+      <c r="M2" s="3"/>
+    </row>
+    <row r="3" spans="1:17" s="1" customFormat="1">
+      <c r="C3" s="4">
+        <v>-12</v>
+      </c>
+      <c r="D3" s="4">
+        <v>-11</v>
+      </c>
+      <c r="E3" s="4">
+        <v>-10</v>
+      </c>
+      <c r="F3" s="4">
+        <v>-9</v>
+      </c>
+      <c r="G3" s="4">
+        <v>-8</v>
+      </c>
+      <c r="H3" s="5">
+        <v>-7</v>
+      </c>
+      <c r="I3" s="5">
+        <v>-6</v>
+      </c>
+      <c r="J3" s="5">
+        <v>-5</v>
+      </c>
+      <c r="K3" s="5">
+        <v>-4</v>
+      </c>
+      <c r="L3" s="5">
+        <v>-3</v>
+      </c>
+      <c r="M3" s="5">
+        <v>-2</v>
+      </c>
+      <c r="N3" s="5">
+        <v>-1</v>
+      </c>
+      <c r="O3" s="5">
+        <v>0</v>
+      </c>
+      <c r="P3" s="6">
+        <v>1</v>
+      </c>
+      <c r="Q3" s="6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" s="1" customFormat="1">
+      <c r="C4" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="I4" s="7"/>
+      <c r="J4" s="7"/>
+      <c r="K4" s="7"/>
+      <c r="L4" s="7"/>
+      <c r="M4" s="7"/>
+      <c r="N4" s="7"/>
+      <c r="O4" s="8"/>
+      <c r="Q4" s="9"/>
+    </row>
+    <row r="5" spans="1:17" s="1" customFormat="1">
+      <c r="A5" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="J5" s="10"/>
+      <c r="K5" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="L5" s="10"/>
+      <c r="M5" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="N5" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="O5" s="10" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" s="1" customFormat="1">
+      <c r="A6" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="J6" s="10"/>
+      <c r="K6" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="L6" s="10"/>
+      <c r="M6" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="N6" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="O6" s="10" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" s="1" customFormat="1">
+      <c r="A7" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="J7" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="K7" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="L7" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="M7" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="10"/>
-      <c r="H2" s="10"/>
-      <c r="I2" s="10"/>
-      <c r="J2" s="10"/>
-    </row>
-    <row r="3" spans="1:15">
-      <c r="C3" s="5">
-        <v>-10</v>
-      </c>
-      <c r="D3" s="5">
-        <v>-9</v>
-      </c>
-      <c r="E3" s="5">
-        <v>-8</v>
-      </c>
-      <c r="F3" s="6">
-        <v>-7</v>
-      </c>
-      <c r="G3" s="6">
-        <v>-6</v>
-      </c>
-      <c r="H3" s="6">
-        <v>-5</v>
-      </c>
-      <c r="I3" s="6">
-        <v>-4</v>
-      </c>
-      <c r="J3" s="6">
-        <v>-3</v>
-      </c>
-      <c r="K3" s="6">
-        <v>-2</v>
-      </c>
-      <c r="L3" s="6">
-        <v>-1</v>
-      </c>
-      <c r="M3" s="6">
+      <c r="N7" s="10"/>
+      <c r="O7" s="10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" s="1" customFormat="1">
+      <c r="A8" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="E8" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="F8" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="G8" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="J8" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="K8" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="L8" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="M8" s="13" t="s">
+        <v>40</v>
+      </c>
+      <c r="N8" s="10"/>
+      <c r="O8" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="N3" s="7">
-        <v>1</v>
-      </c>
-      <c r="O3" s="7">
+    </row>
+    <row r="9" spans="1:17" s="1" customFormat="1">
+      <c r="A9" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="J9" s="10"/>
+      <c r="K9" s="11"/>
+      <c r="L9" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="M9" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="N9" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="O9" s="10" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:15">
-      <c r="C4" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
-      <c r="K4" s="2"/>
-      <c r="L4" s="2"/>
-      <c r="M4" s="8"/>
-      <c r="O4" s="4"/>
-    </row>
-    <row r="5" spans="1:15">
-      <c r="A5" t="s">
-        <v>1</v>
-      </c>
-      <c r="B5" t="s">
+    <row r="10" spans="1:17" s="1" customFormat="1">
+      <c r="A10" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C5" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D5" s="3" t="s">
+      <c r="C10" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="D10" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E10" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="H5" s="3"/>
-      <c r="I5" s="9" t="s">
+      <c r="J10" s="10"/>
+      <c r="K10" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="J5" s="3"/>
-      <c r="K5" s="3" t="s">
+      <c r="L10" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="L5" s="3" t="s">
+      <c r="M10" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="M5" s="3" t="s">
+      <c r="N10" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="O10" s="10" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:15">
-      <c r="A6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" t="s">
-        <v>27</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D6" s="3" t="s">
+    <row r="11" spans="1:17" s="1" customFormat="1">
+      <c r="A11" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="D11" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E11" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="H6" s="3"/>
-      <c r="I6" s="9" t="s">
+      <c r="J11" s="10"/>
+      <c r="K11" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="J6" s="3"/>
-      <c r="K6" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="L6" s="3" t="s">
+      <c r="L11" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="M11" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="M6" s="3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7" spans="1:15">
-      <c r="A7" t="s">
-        <v>17</v>
-      </c>
-      <c r="B7" t="s">
-        <v>27</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="D7" s="3" t="s">
+      <c r="N11" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="O11" s="10" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" s="1" customFormat="1">
+      <c r="A12" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="D12" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="E7" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H7" s="14" t="s">
+      <c r="E12" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="K12" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="L12" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="M12" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="N12" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="O12" s="10" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" s="1" customFormat="1">
+      <c r="A13" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="D13" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="E13" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="H13" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="I13" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="J13" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="K13" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="L13" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="M13" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="N13" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="O13" s="9" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" s="1" customFormat="1">
+      <c r="A14" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="D14" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="E14" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="H14" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="I14" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="J14" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="I7" s="14" t="s">
-        <v>44</v>
-      </c>
-      <c r="J7" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="K7" s="12" t="s">
-        <v>41</v>
-      </c>
-      <c r="L7" s="3"/>
-      <c r="M7" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="8" spans="1:15">
-      <c r="A8" t="s">
-        <v>19</v>
-      </c>
-      <c r="B8" t="s">
-        <v>27</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H8" s="3" t="s">
+      <c r="K14" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="L14" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="I8" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="J8" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="K8" s="12" t="s">
-        <v>41</v>
-      </c>
-      <c r="L8" s="3"/>
-      <c r="M8" s="3" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:15">
-      <c r="A9" t="s">
-        <v>21</v>
-      </c>
-      <c r="B9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="H9" s="3"/>
-      <c r="I9" s="9"/>
-      <c r="J9" s="3" t="s">
+      <c r="M14" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="K9" s="3" t="s">
+      <c r="N14" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="L9" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="M9" s="3" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="10" spans="1:15">
-      <c r="A10" t="s">
-        <v>28</v>
-      </c>
-      <c r="B10" t="s">
-        <v>26</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="H10" s="3"/>
-      <c r="I10" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="J10" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="K10" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="L10" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="M10" s="3" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="11" spans="1:15">
-      <c r="A11" t="s">
-        <v>29</v>
-      </c>
-      <c r="B11" t="s">
-        <v>26</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="H11" s="3"/>
-      <c r="I11" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="J11" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="K11" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="L11" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="M11" s="3" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:15">
-      <c r="A12" t="s">
-        <v>32</v>
-      </c>
-      <c r="B12" t="s">
-        <v>26</v>
-      </c>
-      <c r="C12" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="D12" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E12" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="I12" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="J12" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="K12" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="L12" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="M12" s="3" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="13" spans="1:15">
-      <c r="A13" t="s">
-        <v>36</v>
-      </c>
-      <c r="C13" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D13" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E13" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="F13" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="G13" s="13" t="s">
-        <v>43</v>
-      </c>
-      <c r="H13" s="14" t="s">
-        <v>44</v>
-      </c>
-      <c r="I13" s="14" t="s">
-        <v>44</v>
-      </c>
-      <c r="J13" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="K13" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="L13" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="M13" s="11" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="14" spans="1:15">
-      <c r="A14" t="s">
-        <v>35</v>
-      </c>
-      <c r="C14" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="D14" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E14" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="F14" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="G14" s="13" t="s">
-        <v>43</v>
-      </c>
-      <c r="H14" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="I14" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="J14" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="K14" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="L14" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="M14" s="11" t="s">
+      <c r="O14" s="9" t="s">
         <v>39</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="C2:J2"/>
+    <mergeCell ref="C2:M2"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>